<commit_message>
Nowy wygląd GUI, funkcjonalność dodatkowa, w trakcie rozwoju, na razie nie działa
</commit_message>
<xml_diff>
--- a/karta_postaci.xlsx
+++ b/karta_postaci.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="126">
   <si>
     <t xml:space="preserve">Imię</t>
   </si>
@@ -222,7 +222,7 @@
     <t xml:space="preserve">Przekupstwo</t>
   </si>
   <si>
-    <t xml:space="preserve">język Jałowa Kraina</t>
+    <t xml:space="preserve">Język (Jałowa Kraina)</t>
   </si>
   <si>
     <t xml:space="preserve">15</t>
@@ -300,6 +300,9 @@
     <t xml:space="preserve">Targowanie</t>
   </si>
   <si>
+    <t xml:space="preserve">Język Klasyczny</t>
+  </si>
+  <si>
     <t xml:space="preserve">35</t>
   </si>
   <si>
@@ -318,6 +321,9 @@
     <t xml:space="preserve">Unik</t>
   </si>
   <si>
+    <t xml:space="preserve">Wiedza (Ścieżki Pradawnych)</t>
+  </si>
+  <si>
     <t xml:space="preserve">40</t>
   </si>
   <si>
@@ -334,6 +340,9 @@
   </si>
   <si>
     <t xml:space="preserve">(S)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wiedza (Domena Chaosu)</t>
   </si>
   <si>
     <t xml:space="preserve">45</t>
@@ -1422,13 +1431,13 @@
         <v>27</v>
       </c>
       <c r="P11" s="1" t="n">
-        <v>450</v>
+        <v>185</v>
       </c>
       <c r="Q11" s="1" t="n">
-        <v>1450</v>
+        <v>2260</v>
       </c>
       <c r="R11" s="1" t="n">
-        <v>1900</v>
+        <v>2445</v>
       </c>
       <c r="V11" s="1" t="n">
         <v>500</v>
@@ -1498,7 +1507,7 @@
         <v>8</v>
       </c>
       <c r="J13" s="25" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K13" s="25" t="n">
         <v>0</v>
@@ -1533,7 +1542,7 @@
         <v>50</v>
       </c>
       <c r="J14" s="25" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="K14" s="25" t="n">
         <f aca="false">K12+K13</f>
@@ -1669,10 +1678,10 @@
         <v>31</v>
       </c>
       <c r="I18" s="23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J18" s="39" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="K18" s="41" t="s">
         <v>45</v>
@@ -1681,13 +1690,13 @@
         <v>46</v>
       </c>
       <c r="M18" s="42" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="N18" s="42" t="n">
         <v>10</v>
       </c>
       <c r="O18" s="43" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="Q18" s="30"/>
       <c r="R18" s="30" t="s">
@@ -1713,10 +1722,10 @@
         <v>40</v>
       </c>
       <c r="D19" s="23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E19" s="39" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F19" s="40" t="s">
         <v>50</v>
@@ -2126,13 +2135,23 @@
       <c r="J25" s="39" t="n">
         <v>33</v>
       </c>
-      <c r="K25" s="40"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="N25" s="23"/>
-      <c r="O25" s="39"/>
+      <c r="K25" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="L25" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="M25" s="23" t="n">
+        <v>51</v>
+      </c>
+      <c r="N25" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O25" s="39" t="n">
+        <v>55</v>
+      </c>
       <c r="Q25" s="44" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R25" s="45" t="n">
         <v>120</v>
@@ -2141,21 +2160,21 @@
         <v>80</v>
       </c>
       <c r="V25" s="44" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="W25" s="46" t="s">
         <v>56</v>
       </c>
       <c r="X25" s="45" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>40</v>
@@ -2167,7 +2186,7 @@
         <v>34</v>
       </c>
       <c r="F26" s="40" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G26" s="23" t="s">
         <v>42</v>
@@ -2181,13 +2200,23 @@
       <c r="J26" s="39" t="n">
         <v>38</v>
       </c>
-      <c r="K26" s="40"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="23"/>
-      <c r="N26" s="23"/>
-      <c r="O26" s="39"/>
+      <c r="K26" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="L26" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="M26" s="23" t="n">
+        <v>52</v>
+      </c>
+      <c r="N26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O26" s="39" t="n">
+        <v>52</v>
+      </c>
       <c r="Q26" s="44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="R26" s="45" t="n">
         <v>150</v>
@@ -2196,18 +2225,18 @@
         <v>110</v>
       </c>
       <c r="V26" s="44" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="W26" s="46" t="n">
         <v>1</v>
       </c>
       <c r="X26" s="45" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B27" s="23" t="s">
         <v>44</v>
@@ -2222,10 +2251,10 @@
         <v>31</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H27" s="23" t="n">
         <v>31</v>
@@ -2236,13 +2265,23 @@
       <c r="J27" s="39" t="n">
         <v>31</v>
       </c>
-      <c r="K27" s="40"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="39"/>
+      <c r="K27" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="L27" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="M27" s="23" t="n">
+        <v>53</v>
+      </c>
+      <c r="N27" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" s="39" t="n">
+        <v>53</v>
+      </c>
       <c r="Q27" s="44" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="R27" s="45" t="n">
         <v>190</v>
@@ -2251,21 +2290,21 @@
         <v>140</v>
       </c>
       <c r="V27" s="44" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="W27" s="46" t="n">
         <v>2</v>
       </c>
       <c r="X27" s="45" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>40</v>
@@ -2277,10 +2316,10 @@
         <v>34</v>
       </c>
       <c r="F28" s="40" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H28" s="23" t="n">
         <v>31</v>
@@ -2297,7 +2336,7 @@
       <c r="N28" s="23"/>
       <c r="O28" s="39"/>
       <c r="Q28" s="44" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="R28" s="45" t="n">
         <v>230</v>
@@ -2306,18 +2345,18 @@
         <v>180</v>
       </c>
       <c r="V28" s="44" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="W28" s="46" t="s">
         <v>56</v>
       </c>
       <c r="X28" s="45" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="47" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B29" s="48" t="s">
         <v>46</v>
@@ -2332,7 +2371,7 @@
         <v>47</v>
       </c>
       <c r="F29" s="49" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G29" s="48" t="s">
         <v>51</v>
@@ -2352,7 +2391,7 @@
       <c r="N29" s="23"/>
       <c r="O29" s="39"/>
       <c r="Q29" s="44" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="R29" s="45" t="n">
         <v>280</v>
@@ -2361,18 +2400,18 @@
         <v>220</v>
       </c>
       <c r="V29" s="44" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="W29" s="46" t="n">
         <v>1</v>
       </c>
       <c r="X29" s="45" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="47" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B30" s="48" t="s">
         <v>46</v>
@@ -2387,10 +2426,10 @@
         <v>42</v>
       </c>
       <c r="F30" s="49" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G30" s="48" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H30" s="48" t="n">
         <v>31</v>
@@ -2407,7 +2446,7 @@
       <c r="N30" s="48"/>
       <c r="O30" s="50"/>
       <c r="Q30" s="44" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="R30" s="45" t="n">
         <v>330</v>
@@ -2436,7 +2475,7 @@
       <c r="N31" s="52"/>
       <c r="O31" s="52"/>
       <c r="Q31" s="44" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="R31" s="45" t="n">
         <v>390</v>
@@ -2450,11 +2489,11 @@
     </row>
     <row r="32" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D32" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E32" s="53"/>
       <c r="Q32" s="44" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="R32" s="51" t="n">
         <v>450</v>

</xml_diff>

<commit_message>
Improved functionality and added visibility.
</commit_message>
<xml_diff>
--- a/karta_postaci.xlsx
+++ b/karta_postaci.xlsx
@@ -1275,10 +1275,10 @@
         </is>
       </c>
       <c r="P11" s="58" t="n">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="Q11" s="58" t="n">
-        <v>2290</v>
+        <v>2260</v>
       </c>
       <c r="R11" s="58" t="n">
         <v>2445</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="B13" s="88" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="88" t="n">
         <v>0</v>
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="B14" s="88" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="88" t="n">
         <v>25</v>

</xml_diff>